<commit_message>
[feat/ASP-8019-report-parameters] Added include decommissioned label to report templates
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/uk.xlsx
+++ b/api/templates/critical_errors_by_device/uk.xlsx
@@ -1,36 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED585DD-EBA9-8943-8085-9C465229B040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680"/>
   </bookViews>
   <sheets>
-    <sheet name="Помилки за пристроєм" sheetId="1" r:id="rId1"/>
-    <sheet name="Коди помилок в розрізі пристрої" sheetId="2" r:id="rId2"/>
-    <sheet name="Коди помилок" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Помилки за пристроєм" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Коди помилок в розрізі пристрої" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Коди помилок" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="80">
   <si>
     <t>Помилки за пристроєм</t>
   </si>
@@ -47,18 +33,21 @@
     <t>Сайти: &lt;Sites&gt;</t>
   </si>
   <si>
+    <t>&lt;DecommissionedDevicesLabel&gt;: &lt;DecommissionedDevices&gt;</t>
+  </si>
+  <si>
     <t>&lt;Table&gt;</t>
   </si>
   <si>
     <t>Той самий сайт походження в тесті та зразку</t>
   </si>
   <si>
+    <t>Сайт</t>
+  </si>
+  <si>
     <t>Пристрій</t>
   </si>
   <si>
-    <t>Сайт</t>
-  </si>
-  <si>
     <t>Серіал</t>
   </si>
   <si>
@@ -77,12 +66,12 @@
     <t>Відсоток помилок</t>
   </si>
   <si>
+    <t>&lt;siteName&gt;</t>
+  </si>
+  <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
-    <t>&lt;siteName&gt;</t>
-  </si>
-  <si>
     <t>&lt;serial&gt;</t>
   </si>
   <si>
@@ -128,6 +117,9 @@
     <t>Недійсні результати</t>
   </si>
   <si>
+    <t>Результатів немає</t>
+  </si>
+  <si>
     <t>Всього помилок, недійсних результатів, без результатів</t>
   </si>
   <si>
@@ -164,6 +156,9 @@
     <t>&lt;invalidResults&gt;</t>
   </si>
   <si>
+    <t>&lt;noResults&gt;</t>
+  </si>
+  <si>
     <t>код</t>
   </si>
   <si>
@@ -261,79 +256,80 @@
   </si>
   <si>
     <t>Втрата сигналу, виявлена ​​в кривій ампліфікації</t>
-  </si>
-  <si>
-    <t>Результатів немає</t>
-  </si>
-  <si>
-    <t>&lt;noResults&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm d&quot;, &quot;yyyy;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <charset val="1"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
+      <charset val="1"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="16"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
+      <charset val="1"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
+      <charset val="1"/>
+      <family val="2"/>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <family val="2"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <charset val="1"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -371,18 +367,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
       <diagonal/>
     </border>
     <border>
@@ -443,6 +431,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -455,7 +446,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -465,26 +456,23 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -819,9 +807,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="11.1640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -833,127 +821,131 @@
     <col min="9" max="12" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="21" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
     </row>
-    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-    </row>
-    <row r="8" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="I7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+    </row>
+    <row r="8" ht="33" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="J8" s="7" t="s">
+      <c r="H8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="J8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
+      <c r="L8" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="H9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="I9" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="J9" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L9" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G10" s="1"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G11" s="1"/>
       <c r="H11" s="2"/>
     </row>
@@ -962,14 +954,14 @@
     <mergeCell ref="I7:L7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="9.5"/>
   <cols>
     <col min="1" max="1" width="33.1640625" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -979,9 +971,9 @@
     <col min="1024" max="1024" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="21" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -996,7 +988,7 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1013,7 +1005,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1030,12 +1022,12 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1049,12 +1041,15 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1068,103 +1063,103 @@
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" ht="34.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="14">
         <v>5011</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <v>5007</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="14">
         <v>5006</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="14">
         <v>2008</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="14">
         <v>2005</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="14">
         <v>2037</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="14">
         <v>2025</v>
       </c>
-      <c r="J9" s="16">
+      <c r="J9" s="14">
         <v>2022</v>
       </c>
-      <c r="K9" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="L9" s="16" t="s">
+      <c r="K9" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="M9" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="N9" s="16" t="s">
+      <c r="L9" s="14" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="M9" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="N9" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="18" t="s">
+      <c r="C10" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="D10" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="E10" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="F10" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="I10" s="18" t="s">
+      <c r="G10" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="18" t="s">
+      <c r="H10" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="K10" s="18" t="s">
+      <c r="I10" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="L10" s="18" t="s">
+      <c r="J10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="M10" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="N10" s="18" t="e">
+      <c r="K10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N10" s="16" t="e">
         <f>C10+D10+E10+F10+G10+H10+I10+J10+K10+L10+M10</f>
         <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>
@@ -1173,315 +1168,315 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="9.5"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="120.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13">
+    <row r="1" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
         <v>1001</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="B2" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="18">
         <v>1002</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="B3" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
         <v>1004</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="C4" s="18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
         <v>1005</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="B5" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
         <v>1006</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="B6" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
         <v>1007</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="B7" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
         <v>1017</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="B8" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
         <v>1018</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="B9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
         <v>2003</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="B10" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
         <v>2005</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="B11" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
         <v>2008</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="13" t="s">
+      <c r="B12" s="18" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="C12" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="18">
         <v>2009</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="B13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="18">
         <v>2011</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="13">
+      <c r="B14" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" ht="30.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="18">
         <v>2014</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="13">
+      <c r="B15" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="18">
         <v>2016</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="13" t="s">
+      <c r="B16" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
+        <v>2018</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="13">
-        <v>2018</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="13">
+      <c r="C17" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="18">
         <v>2022</v>
       </c>
-      <c r="B18" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="13" t="s">
+      <c r="B18" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="18">
+        <v>2025</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="18">
+        <v>2032</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="18">
+        <v>2034</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="18">
+        <v>2037</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="18">
+        <v>4010</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" ht="30.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
+        <v>4017</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="18" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="13">
-        <v>2025</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="13">
-        <v>2032</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="13">
-        <v>2034</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="13">
-        <v>2037</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="13">
-        <v>4010</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="13">
-        <v>4017</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="13">
+    <row r="25" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="18">
         <v>5006</v>
       </c>
-      <c r="B25" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="13">
+      <c r="B25" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="18">
         <v>5007</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="13">
+      <c r="B26" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="18">
         <v>5011</v>
       </c>
-      <c r="B27" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="13" t="s">
+      <c r="B27" s="18" t="s">
         <v>76</v>
       </c>
+      <c r="C27" s="18" t="s">
+        <v>79</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>

</xml_diff>